<commit_message>
CI Reports [2026-07-01 09:03]: CreateTicket — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Feature Reports/CreateTicket.xlsx
+++ b/Test Execution Report_Git/Feature Reports/CreateTicket.xlsx
@@ -468,7 +468,7 @@
         <v>Remarks</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
         <v>TC-CT-001</v>
       </c>
@@ -488,16 +488,24 @@
         <v>API</v>
       </c>
       <c r="G2" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H2" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>Application accessible at http://customerportal.dev-ts.online; sajith_xyz account active</v>
+      </c>
+      <c r="H2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Login as sajith_xyz / User@123
+2. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+3. Select project: PRJ0008 - YSG Inventory
+4. Click the 'New' ticket type chip
+5. Click the 'Backend' platform chip
+6. Enter description (112 chars): 'This is a test ticket created by automated QA testing...'
+7. Click Submit Ticket button
+8. Click 'Yes, Submit' on the confirmation dialog
+9. Observe success dialog and redirect</v>
       </c>
       <c r="I2" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Project: PRJ0008 - YSG Inventory | Type: New | Platform: Backend | Desc: 112-char valid text</v>
       </c>
       <c r="J2" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>'Ticket Submitted!' success dialog shown; redirected to /Ticket/Index after clicking 'Great!'</v>
       </c>
       <c r="K2" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -518,7 +526,7 @@
         <v/>
       </c>
     </row>
-    <row r="3">
+    <row r="3" xml:space="preserve">
       <c r="A3" t="str">
         <v>TC-CT-002</v>
       </c>
@@ -538,16 +546,22 @@
         <v>API</v>
       </c>
       <c r="G3" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H3" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select project: PRJ0021 - YSG Loyalty
+3. Enter Page/Screen Name: 'Dashboard'
+4. Click 'Improvement' type chip
+5. Click 'General' platform chip
+6. Enter description: 'Minimal valid ticket with exactly fifteen chars.'
+7. Click Submit Ticket → 'Yes, Submit'</v>
       </c>
       <c r="I3" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Project: PRJ0021 - YSG Loyalty | Page Name: Dashboard | Type: Improvement | Platform: General</v>
       </c>
       <c r="J3" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>Ticket submitted successfully including Page/Screen Name; 'Ticket Submitted!' dialog shown</v>
       </c>
       <c r="K3" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -568,7 +582,7 @@
         <v/>
       </c>
     </row>
-    <row r="4">
+    <row r="4" xml:space="preserve">
       <c r="A4" t="str">
         <v>TC-CT-003</v>
       </c>
@@ -588,16 +602,19 @@
         <v>Auto</v>
       </c>
       <c r="G4" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H4" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Click each type chip: New, Improvement, System Issue, Operational Issue, SCR, Not Feasible
+3. Verify each chip toggles to selected state (CSS class change) after click
+4. Deselect each chip after verification</v>
       </c>
       <c r="I4" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Chips: New | Improvement | System Issue | Operational Issue | SCR | Not Feasible</v>
       </c>
       <c r="J4" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>Each of the 6 type chips toggles to selected state when clicked; deselects on second click</v>
       </c>
       <c r="K4" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -618,7 +635,7 @@
         <v/>
       </c>
     </row>
-    <row r="5">
+    <row r="5" xml:space="preserve">
       <c r="A5" t="str">
         <v>TC-CT-004</v>
       </c>
@@ -638,16 +655,19 @@
         <v>Auto</v>
       </c>
       <c r="G5" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H5" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Click each platform chip: Backend, SFA Web Service, Android, Web Service, Integration, General, Testing
+3. Verify each chip toggles to selected state
+4. Deselect each chip after verification</v>
       </c>
       <c r="I5" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Chips: Backend | SFA Web Service | Android | Web Service | Integration | General | Testing</v>
       </c>
       <c r="J5" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>All 7 platform chips toggle to selected state when clicked</v>
       </c>
       <c r="K5" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -668,7 +688,7 @@
         <v/>
       </c>
     </row>
-    <row r="6">
+    <row r="6" xml:space="preserve">
       <c r="A6" t="str">
         <v>TC-CT-005</v>
       </c>
@@ -688,16 +708,22 @@
         <v>API</v>
       </c>
       <c r="G6" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H6" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Enter Page/Screen Name: 'Test Page'
+3. Enter Description: 'Filled description'
+4. Click the Reset button
+5. Verify 'Reset Form?' confirmation dialog appears
+6. Click the confirm/Yes button
+7. Verify all fields are cleared</v>
       </c>
       <c r="I6" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Reset confirmation dialog; all fields post-reset</v>
       </c>
       <c r="J6" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>'Reset Form?' dialog shown; after confirm: desc='', pageName='', counter='0/2000', project=''</v>
       </c>
       <c r="K6" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -718,7 +744,7 @@
         <v/>
       </c>
     </row>
-    <row r="7">
+    <row r="7" xml:space="preserve">
       <c r="A7" t="str">
         <v>TC-CT-006</v>
       </c>
@@ -738,16 +764,20 @@
         <v>API</v>
       </c>
       <c r="G7" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H7" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Observe description counter shows '0 / 2000'
+3. Click in the Description textarea
+4. Type: 'Testing counter update!'
+5. Observe the counter value below the textarea</v>
       </c>
       <c r="I7" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Text: 'Testing counter update!' (23 chars)</v>
       </c>
       <c r="J7" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>Counter starts at '0 / 2000'; updates dynamically to current character count as user types</v>
       </c>
       <c r="K7" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -768,7 +798,7 @@
         <v/>
       </c>
     </row>
-    <row r="8">
+    <row r="8" xml:space="preserve">
       <c r="A8" t="str">
         <v>TC-CT-007</v>
       </c>
@@ -788,16 +818,24 @@
         <v>Auto</v>
       </c>
       <c r="G8" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H8" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>Application accessible at http://customerportal.dev-ts.online; sajith_xyz account active</v>
+      </c>
+      <c r="H8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Login as sajith_xyz
+2. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+3. Verify page title = 'Create Ticket - Support'
+4. Verify h1 heading = 'Create New Ticket'
+5. Verify Submit Ticket button is visible
+6. Verify Reset button is visible
+7. Verify #txtDescription textarea is visible
+8. Verify #descCount counter shows '0 / 2000'
+9. Verify #txtPageName input is visible</v>
       </c>
       <c r="I8" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>URL: http://customerportal.dev-ts.online/Ticket/Create</v>
       </c>
       <c r="J8" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>title='Create Ticket - Support'; h1='Create New Ticket'; Submit/Reset/Desc/Counter/PageName all visible; counter='0/2000'</v>
       </c>
       <c r="K8" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -818,7 +856,7 @@
         <v/>
       </c>
     </row>
-    <row r="9">
+    <row r="9" xml:space="preserve">
       <c r="A9" t="str">
         <v>TC-CT-008</v>
       </c>
@@ -838,16 +876,21 @@
         <v>API</v>
       </c>
       <c r="G9" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H9" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select Ticket Type: New
+3. Select Platform: Backend
+4. Enter valid description (&gt;15 chars)
+5. Leave Project field empty
+6. Click Submit Ticket</v>
       </c>
       <c r="I9" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Project: (empty) | Type: New | Platform: Backend | Desc: valid</v>
       </c>
       <c r="J9" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>'Missing Information' dialog: 'Please provide the following mandatory details: Project'</v>
       </c>
       <c r="K9" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -868,7 +911,7 @@
         <v/>
       </c>
     </row>
-    <row r="10">
+    <row r="10" xml:space="preserve">
       <c r="A10" t="str">
         <v>TC-CT-009</v>
       </c>
@@ -888,16 +931,21 @@
         <v>API</v>
       </c>
       <c r="G10" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H10" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select Project: PRJ0008 - YSG Inventory
+3. Select Platform: Backend
+4. Enter valid description (&gt;15 chars)
+5. Leave Ticket Type unselected
+6. Click Submit Ticket</v>
       </c>
       <c r="I10" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Project: PRJ0008 | Type: (none) | Platform: Backend | Desc: valid</v>
       </c>
       <c r="J10" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>'Missing Information' dialog: 'Please provide: Ticket Type'</v>
       </c>
       <c r="K10" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -918,7 +966,7 @@
         <v/>
       </c>
     </row>
-    <row r="11">
+    <row r="11" xml:space="preserve">
       <c r="A11" t="str">
         <v>TC-CT-010</v>
       </c>
@@ -938,16 +986,20 @@
         <v>API</v>
       </c>
       <c r="G11" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H11" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select Project and Ticket Type: New
+3. Enter valid description
+4. Leave Platform unselected
+5. Click Submit Ticket</v>
       </c>
       <c r="I11" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Project: PRJ0008 | Type: New | Platform: (none) | Desc: valid</v>
       </c>
       <c r="J11" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>'Missing Information' dialog: 'Please provide: Platform'</v>
       </c>
       <c r="K11" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -968,7 +1020,7 @@
         <v/>
       </c>
     </row>
-    <row r="12">
+    <row r="12" xml:space="preserve">
       <c r="A12" t="str">
         <v>TC-CT-011</v>
       </c>
@@ -988,16 +1040,19 @@
         <v>API</v>
       </c>
       <c r="G12" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H12" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select Project, Ticket Type: New, Platform: Backend
+3. Leave Description field empty
+4. Click Submit Ticket</v>
       </c>
       <c r="I12" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Project: PRJ0008 | Type: New | Platform: Backend | Desc: (empty)</v>
       </c>
       <c r="J12" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>'Missing Information' dialog: 'Please provide: Description (min 15 chars)'</v>
       </c>
       <c r="K12" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1018,7 +1073,7 @@
         <v/>
       </c>
     </row>
-    <row r="13">
+    <row r="13" xml:space="preserve">
       <c r="A13" t="str">
         <v>TC-CT-012</v>
       </c>
@@ -1038,16 +1093,19 @@
         <v>API</v>
       </c>
       <c r="G13" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H13" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select all required fields
+3. Enter description: '14charsonly!!!' (14 chars)
+4. Click Submit Ticket</v>
       </c>
       <c r="I13" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Description: '14charsonly!!!' — 14 characters (below 15 minimum)</v>
       </c>
       <c r="J13" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>'Missing Information' → 'Description (min 15 chars)'; form not submitted</v>
       </c>
       <c r="K13" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1068,7 +1126,7 @@
         <v/>
       </c>
     </row>
-    <row r="14">
+    <row r="14" xml:space="preserve">
       <c r="A14" t="str">
         <v>TC-CT-013</v>
       </c>
@@ -1088,16 +1146,18 @@
         <v>Unit</v>
       </c>
       <c r="G14" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H14" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create (all fields empty on load)
+2. Click Submit Ticket immediately without filling any field
+3. Observe validation dialog</v>
       </c>
       <c r="I14" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>All fields: (empty)</v>
       </c>
       <c r="J14" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>'Missing Information' dialog listing all 4 missing fields: Project, Ticket Type, Description (min 15 chars), Platform</v>
       </c>
       <c r="K14" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1118,7 +1178,7 @@
         <v/>
       </c>
     </row>
-    <row r="15">
+    <row r="15" xml:space="preserve">
       <c r="A15" t="str">
         <v>TC-CT-014</v>
       </c>
@@ -1138,16 +1198,20 @@
         <v>API</v>
       </c>
       <c r="G15" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H15" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select all required fields
+3. Enter exactly 15-character description: 'Test15CharsOnly'
+4. Verify counter shows '15 / 2000'
+5. Click Submit Ticket</v>
       </c>
       <c r="I15" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Description: 'Test15CharsOnly' — exactly 15 characters</v>
       </c>
       <c r="J15" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>15-char description accepted; counter='15/2000'; 'Submit Ticket?' confirmation dialog shown</v>
       </c>
       <c r="K15" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1168,7 +1232,7 @@
         <v/>
       </c>
     </row>
-    <row r="16">
+    <row r="16" xml:space="preserve">
       <c r="A16" t="str">
         <v>TC-CT-015</v>
       </c>
@@ -1188,16 +1252,19 @@
         <v>API</v>
       </c>
       <c r="G16" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H16" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select all required fields
+3. Enter exactly 14-character description: '14charsonly!!!'
+4. Click Submit Ticket</v>
       </c>
       <c r="I16" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Description: '14charsonly!!!' — exactly 14 characters</v>
       </c>
       <c r="J16" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>Validation error shown; 14-char description rejected; form not submitted</v>
       </c>
       <c r="K16" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1218,7 +1285,7 @@
         <v/>
       </c>
     </row>
-    <row r="17">
+    <row r="17" xml:space="preserve">
       <c r="A17" t="str">
         <v>TC-CT-016</v>
       </c>
@@ -1238,16 +1305,20 @@
         <v>API</v>
       </c>
       <c r="G17" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H17" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select all required fields
+3. Enter exactly 2000 'A' characters in Description
+4. Verify counter shows '2000 / 2000'
+5. Click Submit Ticket</v>
       </c>
       <c r="I17" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Description: 'A'×2000 — exactly 2000 characters</v>
       </c>
       <c r="J17" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>Counter='2000/2000'; form accepts 2000-char description; 'Submit Ticket?' dialog shown</v>
       </c>
       <c r="K17" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1268,7 +1339,7 @@
         <v/>
       </c>
     </row>
-    <row r="18">
+    <row r="18" xml:space="preserve">
       <c r="A18" t="str">
         <v>TC-CT-017</v>
       </c>
@@ -1288,16 +1359,21 @@
         <v>API</v>
       </c>
       <c r="G18" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H18" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select all required fields
+3. Enter 2001 'A' characters in Description
+4. Observe counter value
+5. Click Submit Ticket
+6. Observe whether submission is blocked</v>
       </c>
       <c r="I18" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Description: 'A'×2001 — 1 char over the 2000 max shown in UI</v>
       </c>
       <c r="J18" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>Input truncated to 2000 chars OR submission blocked with validation error; counter should not exceed 2000/2000</v>
       </c>
       <c r="K18" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1318,7 +1394,7 @@
         <v/>
       </c>
     </row>
-    <row r="19">
+    <row r="19" xml:space="preserve">
       <c r="A19" t="str">
         <v>TC-CT-018</v>
       </c>
@@ -1338,16 +1414,19 @@
         <v>API</v>
       </c>
       <c r="G19" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H19" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select all required fields with valid description
+3. Enter 300-character string in Page/Screen Name field
+4. Click Submit Ticket → confirm</v>
       </c>
       <c r="I19" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Page/Screen Name: 'A'×300 (300 characters)</v>
       </c>
       <c r="J19" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>App handles 300-char page name; no crash or 500 error; ticket submitted successfully</v>
       </c>
       <c r="K19" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1368,7 +1447,7 @@
         <v/>
       </c>
     </row>
-    <row r="20">
+    <row r="20" xml:space="preserve">
       <c r="A20" t="str">
         <v>TC-CT-019</v>
       </c>
@@ -1388,22 +1467,25 @@
         <v>Auto</v>
       </c>
       <c r="G20" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H20" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>No active session (HttpOnly cookies cleared)</v>
+      </c>
+      <c r="H20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Clear all session cookies (page.context().clearCookies())
+2. Navigate directly to http://customerportal.dev-ts.online/Ticket/Create
+3. Observe redirect behaviour
+4. Verify URL changes to /Account/Login</v>
       </c>
       <c r="I20" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Session: cleared | Direct target URL: http://customerportal.dev-ts.online/Ticket/Create</v>
       </c>
       <c r="J20" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>Unauthenticated direct access blocked; redirected to /Account/Login; auth guard active</v>
       </c>
       <c r="K20" t="str">
-        <v>TypeError: url.includes is not a function</v>
+        <v>All assertions passed via Playwright</v>
       </c>
       <c r="L20" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="M20" t="str">
         <v>Playwright Automation</v>
@@ -1418,7 +1500,7 @@
         <v/>
       </c>
     </row>
-    <row r="21">
+    <row r="21" xml:space="preserve">
       <c r="A21" t="str">
         <v>TC-CT-020</v>
       </c>
@@ -1438,16 +1520,20 @@
         <v>API</v>
       </c>
       <c r="G21" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H21" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select all required fields
+3. Enter SQL injection payload in Description
+4. Click Submit Ticket → confirm
+5. Verify no SQL error or server crash</v>
       </c>
       <c r="I21" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Description: ' OR 1=1 --; DROP TABLE tickets; SELECT * FROM users;</v>
       </c>
       <c r="J21" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>SQL payload submitted safely; no SQL error or data leak; no server crash; ticket submitted normally</v>
       </c>
       <c r="K21" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1468,7 +1554,7 @@
         <v/>
       </c>
     </row>
-    <row r="22">
+    <row r="22" xml:space="preserve">
       <c r="A22" t="str">
         <v>TC-CT-021</v>
       </c>
@@ -1488,16 +1574,21 @@
         <v>API</v>
       </c>
       <c r="G22" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H22" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select all required fields
+3. Enter XSS payload in Description: &lt;script&gt;alert('xss')&lt;/script&gt;
+4. Override window.alert to detect execution
+5. Click Submit Ticket → confirm
+6. Verify no JS alert dialog fires</v>
       </c>
       <c r="I22" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Description: &lt;script&gt;alert('xss')&lt;/script&gt;</v>
       </c>
       <c r="J22" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>XSS payload submitted as plain text; no JS alert fires; input not executed in browser</v>
       </c>
       <c r="K22" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1518,7 +1609,7 @@
         <v/>
       </c>
     </row>
-    <row r="23">
+    <row r="23" xml:space="preserve">
       <c r="A23" t="str">
         <v>TC-CT-022</v>
       </c>
@@ -1538,16 +1629,20 @@
         <v>API</v>
       </c>
       <c r="G23" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H23" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select all required fields
+3. Enter HTML injection payload in Description: &lt;img src=x onerror=alert(1)&gt;
+4. Override window.alert to detect execution
+5. Click Submit Ticket → confirm</v>
       </c>
       <c r="I23" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Description: &lt;img src=x onerror=alert(1)&gt;</v>
       </c>
       <c r="J23" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>HTML injection not executed; no alert fires; payload stored as plain text</v>
       </c>
       <c r="K23" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1568,7 +1663,7 @@
         <v/>
       </c>
     </row>
-    <row r="24">
+    <row r="24" xml:space="preserve">
       <c r="A24" t="str">
         <v>TC-CT-023</v>
       </c>
@@ -1588,16 +1683,20 @@
         <v>API</v>
       </c>
       <c r="G24" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H24" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select all required fields with valid description
+3. Enter XSS payload in Page/Screen Name: &lt;script&gt;alert('xss')&lt;/script&gt;
+4. Override window.alert to detect execution
+5. Click Submit Ticket → confirm</v>
       </c>
       <c r="I24" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Page/Screen Name: &lt;script&gt;alert('xss')&lt;/script&gt;</v>
       </c>
       <c r="J24" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>XSS in page name not executed; no JS alert fires</v>
       </c>
       <c r="K24" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1618,7 +1717,7 @@
         <v/>
       </c>
     </row>
-    <row r="25">
+    <row r="25" xml:space="preserve">
       <c r="A25" t="str">
         <v>TC-CT-024</v>
       </c>
@@ -1638,16 +1737,21 @@
         <v>API</v>
       </c>
       <c r="G25" t="str">
-        <v>Application accessible at http://customerportal.dev-ts.online; user sajith_xyz active</v>
-      </c>
-      <c r="H25" t="str">
-        <v>(See Playwright spec: tests/createticket.spec.js)</v>
+        <v>User logged in as sajith_xyz; on Create Ticket page (/Ticket/Create)</v>
+      </c>
+      <c r="H25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to http://customerportal.dev-ts.online/Ticket/Create
+2. Select Project, Type, Platform; enter description
+3. Click Reset button
+4. Verify 'Reset Form?' dialog appears
+5. Click 'Wait, let me check' / cancel button
+6. Verify all previously entered fields are still populated</v>
       </c>
       <c r="I25" t="str">
-        <v>See test-data/createticketData.js</v>
+        <v>Description: 'This text should remain after cancel reset click test.'</v>
       </c>
       <c r="J25" t="str">
-        <v>Test assertions pass per spec definition</v>
+        <v>'Reset Form?' dialog dismisses on cancel; form fields remain unchanged; no data lost</v>
       </c>
       <c r="K25" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1677,7 +1781,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P24"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -1770,12 +1874,13 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-001
-3. Observe failure</v>
+        <v xml:space="preserve">1. Login and navigate to /Ticket/Create
+2. Fill all required fields with valid data
+3. Click Submit Ticket → 'Yes, Submit'
+4. Observe — 'Ticket Submitted!' dialog should appear</v>
       </c>
       <c r="I2" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>'Ticket Submitted!' success dialog shown; redirected to /Ticket/Index after clicking 'Great!'</v>
       </c>
       <c r="J2" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1822,12 +1927,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-002
-3. Observe failure</v>
+        <v xml:space="preserve">1. Fill all required fields + Page/Screen Name
+2. Click Submit Ticket → 'Yes, Submit'
+3. Observe success dialog</v>
       </c>
       <c r="I3" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>Ticket submitted successfully including Page/Screen Name; 'Ticket Submitted!' dialog shown</v>
       </c>
       <c r="J3" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1874,12 +1979,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-003
-3. Observe failure</v>
+        <v xml:space="preserve">1. Click each type chip in turn
+2. Verify selected CSS class applied
+3. Note which chip(s) fail to select</v>
       </c>
       <c r="I4" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>Each of the 6 type chips toggles to selected state when clicked; deselects on second click</v>
       </c>
       <c r="J4" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1926,12 +2031,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H5" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-004
-3. Observe failure</v>
+        <v xml:space="preserve">1. Click each platform chip
+2. Verify selected state
+3. Note which chip(s) fail to select</v>
       </c>
       <c r="I5" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>All 7 platform chips toggle to selected state when clicked</v>
       </c>
       <c r="J5" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -1978,12 +2083,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-005
-3. Observe failure</v>
+        <v xml:space="preserve">1. Fill some fields then click Reset
+2. Confirm in the dialog
+3. Observe which fields are not cleared</v>
       </c>
       <c r="I6" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>'Reset Form?' dialog shown; after confirm: desc='', pageName='', counter='0/2000', project=''</v>
       </c>
       <c r="J6" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2030,12 +2135,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H7" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-006
-3. Observe failure</v>
+        <v xml:space="preserve">1. Type in description field
+2. Check if counter updates in real-time
+3. Note if counter remains static</v>
       </c>
       <c r="I7" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>Counter starts at '0 / 2000'; updates dynamically to current character count as user types</v>
       </c>
       <c r="J7" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2082,12 +2187,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H8" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-007
-3. Observe failure</v>
+        <v xml:space="preserve">1. Navigate to /Ticket/Create
+2. Check for missing or incorrect UI elements
+3. Note which elements are not visible</v>
       </c>
       <c r="I8" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>title='Create Ticket - Support'; h1='Create New Ticket'; Submit/Reset/Desc/Counter/PageName all visible; counter='0/2000'</v>
       </c>
       <c r="J8" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2134,12 +2239,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H9" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-008
-3. Observe failure</v>
+        <v xml:space="preserve">1. Fill type/platform/desc but leave project empty
+2. Click Submit Ticket
+3. Observe if validation error appears for Project</v>
       </c>
       <c r="I9" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>'Missing Information' dialog: 'Please provide the following mandatory details: Project'</v>
       </c>
       <c r="J9" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2186,12 +2291,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H10" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-009
-3. Observe failure</v>
+        <v xml:space="preserve">1. Fill project/platform/desc but leave ticket type empty
+2. Click Submit
+3. Check validation</v>
       </c>
       <c r="I10" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>'Missing Information' dialog: 'Please provide: Ticket Type'</v>
       </c>
       <c r="J10" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2238,12 +2343,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H11" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-010
-3. Observe failure</v>
+        <v xml:space="preserve">1. Fill project/type/desc but leave platform empty
+2. Click Submit
+3. Check validation</v>
       </c>
       <c r="I11" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>'Missing Information' dialog: 'Please provide: Platform'</v>
       </c>
       <c r="J11" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2290,12 +2395,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H12" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-011
-3. Observe failure</v>
+        <v xml:space="preserve">1. Fill project/type/platform but leave description empty
+2. Click Submit
+3. Check validation</v>
       </c>
       <c r="I12" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>'Missing Information' dialog: 'Please provide: Description (min 15 chars)'</v>
       </c>
       <c r="J12" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2342,12 +2447,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H13" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-012
-3. Observe failure</v>
+        <v xml:space="preserve">1. Enter 14-char description
+2. Click Submit
+3. Check if below-minimum is accepted</v>
       </c>
       <c r="I13" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>'Missing Information' → 'Description (min 15 chars)'; form not submitted</v>
       </c>
       <c r="J13" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2394,12 +2499,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H14" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-013
-3. Observe failure</v>
+        <v xml:space="preserve">1. Navigate to form
+2. Click Submit without filling anything
+3. Check all validations shown</v>
       </c>
       <c r="I14" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>'Missing Information' dialog listing all 4 missing fields: Project, Ticket Type, Description (min 15 chars), Platform</v>
       </c>
       <c r="J14" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2446,12 +2551,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H15" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-014
-3. Observe failure</v>
+        <v xml:space="preserve">1. Enter exactly 15 chars
+2. Click Submit
+3. Check if minimum boundary is accepted</v>
       </c>
       <c r="I15" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>15-char description accepted; counter='15/2000'; 'Submit Ticket?' confirmation dialog shown</v>
       </c>
       <c r="J15" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2498,12 +2603,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H16" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-015
-3. Observe failure</v>
+        <v xml:space="preserve">1. Enter 14-char description
+2. Click Submit
+3. Check if below-min boundary is rejected</v>
       </c>
       <c r="I16" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>Validation error shown; 14-char description rejected; form not submitted</v>
       </c>
       <c r="J16" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2550,12 +2655,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H17" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-016
-3. Observe failure</v>
+        <v xml:space="preserve">1. Enter 2000 chars
+2. Click Submit
+3. Check max boundary acceptance</v>
       </c>
       <c r="I17" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>Counter='2000/2000'; form accepts 2000-char description; 'Submit Ticket?' dialog shown</v>
       </c>
       <c r="J17" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2602,12 +2707,14 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H18" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-017
-3. Observe failure</v>
+        <v xml:space="preserve">1. Enter 2001 chars in description
+2. Note counter shows '2001 / 2000'
+3. Click Submit Ticket
+4. Observe — 'Submit Ticket?' confirm appears; ticket submits with 2001 chars
+5. No server-side max-length enforcement present</v>
       </c>
       <c r="I18" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>Input truncated to 2000 chars OR submission blocked with validation error; counter should not exceed 2000/2000</v>
       </c>
       <c r="J18" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2654,12 +2761,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H19" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-018
-3. Observe failure</v>
+        <v xml:space="preserve">1. Enter 300-char page name
+2. Submit ticket
+3. Check for crash or 500 error</v>
       </c>
       <c r="I19" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>App handles 300-char page name; no crash or 500 error; ticket submitted successfully</v>
       </c>
       <c r="J19" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2688,13 +2795,13 @@
         <v>BUG-CREATETICKET-019</v>
       </c>
       <c r="B20" t="str">
-        <v>Unauthenticated access redirects to login</v>
+        <v>SQL injection in description handled safely</v>
       </c>
       <c r="C20" t="str">
         <v>CreateTicket</v>
       </c>
       <c r="D20" t="str">
-        <v>TC-CT-019</v>
+        <v>TC-CT-020</v>
       </c>
       <c r="E20" t="str">
         <v>High</v>
@@ -2706,12 +2813,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H20" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-019
-3. Observe failure</v>
+        <v xml:space="preserve">1. Enter SQL injection in description
+2. Submit
+3. Check for SQL errors or 500</v>
       </c>
       <c r="I20" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>SQL payload submitted safely; no SQL error or data leak; no server crash; ticket submitted normally</v>
       </c>
       <c r="J20" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2740,13 +2847,13 @@
         <v>BUG-CREATETICKET-020</v>
       </c>
       <c r="B21" t="str">
-        <v>SQL injection in description handled safely</v>
+        <v>XSS payload in description does not execute</v>
       </c>
       <c r="C21" t="str">
         <v>CreateTicket</v>
       </c>
       <c r="D21" t="str">
-        <v>TC-CT-020</v>
+        <v>TC-CT-021</v>
       </c>
       <c r="E21" t="str">
         <v>High</v>
@@ -2758,12 +2865,12 @@
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H21" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-020
-3. Observe failure</v>
+        <v xml:space="preserve">1. Enter &lt;script&gt;alert('xss')&lt;/script&gt;
+2. Submit
+3. Check if alert fires</v>
       </c>
       <c r="I21" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>XSS payload submitted as plain text; no JS alert fires; input not executed in browser</v>
       </c>
       <c r="J21" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2792,30 +2899,30 @@
         <v>BUG-CREATETICKET-021</v>
       </c>
       <c r="B22" t="str">
-        <v>XSS payload in description does not execute</v>
+        <v>HTML injection in description is sanitised</v>
       </c>
       <c r="C22" t="str">
         <v>CreateTicket</v>
       </c>
       <c r="D22" t="str">
-        <v>TC-CT-021</v>
+        <v>TC-CT-022</v>
       </c>
       <c r="E22" t="str">
-        <v>High</v>
+        <v>Low</v>
       </c>
       <c r="F22" t="str">
-        <v>P2</v>
+        <v>P3</v>
       </c>
       <c r="G22" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H22" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-021
-3. Observe failure</v>
+        <v xml:space="preserve">1. Enter &lt;img src=x onerror=alert(1)&gt; in description
+2. Submit
+3. Check if alert fires</v>
       </c>
       <c r="I22" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>HTML injection not executed; no alert fires; payload stored as plain text</v>
       </c>
       <c r="J22" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2844,30 +2951,30 @@
         <v>BUG-CREATETICKET-022</v>
       </c>
       <c r="B23" t="str">
-        <v>HTML injection in description is sanitised</v>
+        <v>XSS payload in Page/Screen Name does not execute</v>
       </c>
       <c r="C23" t="str">
         <v>CreateTicket</v>
       </c>
       <c r="D23" t="str">
-        <v>TC-CT-022</v>
+        <v>TC-CT-023</v>
       </c>
       <c r="E23" t="str">
-        <v>Low</v>
+        <v>High</v>
       </c>
       <c r="F23" t="str">
-        <v>P3</v>
+        <v>P2</v>
       </c>
       <c r="G23" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H23" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-022
-3. Observe failure</v>
+        <v xml:space="preserve">1. Enter XSS payload in page name
+2. Submit
+3. Check if alert fires</v>
       </c>
       <c r="I23" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>XSS in page name not executed; no JS alert fires</v>
       </c>
       <c r="J23" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2896,30 +3003,31 @@
         <v>BUG-CREATETICKET-023</v>
       </c>
       <c r="B24" t="str">
-        <v>XSS payload in Page/Screen Name does not execute</v>
+        <v>Cancel Reset dialog retains all form fields</v>
       </c>
       <c r="C24" t="str">
         <v>CreateTicket</v>
       </c>
       <c r="D24" t="str">
-        <v>TC-CT-023</v>
+        <v>TC-CT-024</v>
       </c>
       <c r="E24" t="str">
-        <v>High</v>
+        <v>Low</v>
       </c>
       <c r="F24" t="str">
-        <v>P2</v>
+        <v>P3</v>
       </c>
       <c r="G24" t="str">
         <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
       </c>
       <c r="H24" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-023
-3. Observe failure</v>
+        <v xml:space="preserve">1. Fill form
+2. Click Reset
+3. Click Cancel
+4. Check if fields are retained</v>
       </c>
       <c r="I24" t="str">
-        <v>All Playwright assertions should pass</v>
+        <v>'Reset Form?' dialog dismisses on cancel; form fields remain unchanged; no data lost</v>
       </c>
       <c r="J24" t="str">
         <v>TypeError: url.includes is not a function</v>
@@ -2943,61 +3051,9 @@
         <v/>
       </c>
     </row>
-    <row r="25" xml:space="preserve">
-      <c r="A25" t="str">
-        <v>BUG-CREATETICKET-024</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Cancel Reset dialog retains all form fields</v>
-      </c>
-      <c r="C25" t="str">
-        <v>CreateTicket</v>
-      </c>
-      <c r="D25" t="str">
-        <v>TC-CT-024</v>
-      </c>
-      <c r="E25" t="str">
-        <v>Low</v>
-      </c>
-      <c r="F25" t="str">
-        <v>P3</v>
-      </c>
-      <c r="G25" t="str">
-        <v>http://customerportal.dev-ts.online | Chrome | Windows | Headless</v>
-      </c>
-      <c r="H25" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to CreateTicket feature
-2. Execute: TC-CT-024
-3. Observe failure</v>
-      </c>
-      <c r="I25" t="str">
-        <v>All Playwright assertions should pass</v>
-      </c>
-      <c r="J25" t="str">
-        <v>TypeError: url.includes is not a function</v>
-      </c>
-      <c r="K25" t="str">
-        <v>New</v>
-      </c>
-      <c r="L25" t="str">
-        <v>Playwright Automation</v>
-      </c>
-      <c r="M25" t="str">
-        <v>01 Jul 2026</v>
-      </c>
-      <c r="N25" t="str">
-        <v/>
-      </c>
-      <c r="O25" t="str">
-        <v>Not Run</v>
-      </c>
-      <c r="P25" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CI Reports [2026-07-01 15:59]: CreateTicket — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Feature Reports/CreateTicket.xlsx
+++ b/Test Execution Report_Git/Feature Reports/CreateTicket.xlsx
@@ -749,7 +749,7 @@
         <v>TC-CT-006</v>
       </c>
       <c r="B7" t="str">
-        <v>Character counter updates dynamically as user types</v>
+        <v>Character counter updates dynamically</v>
       </c>
       <c r="C7" t="str">
         <v>CreateTicket</v>
@@ -2117,7 +2117,7 @@
         <v>BUG-CREATETICKET-006</v>
       </c>
       <c r="B7" t="str">
-        <v>Character counter updates dynamically as user types</v>
+        <v>Character counter updates dynamically</v>
       </c>
       <c r="C7" t="str">
         <v>CreateTicket</v>

</xml_diff>